<commit_message>
Correct Dreamcare customer name
</commit_message>
<xml_diff>
--- a/고객관리_연락처기준.xlsx
+++ b/고객관리_연락처기준.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="고객관리" sheetId="1" r:id="R1cb3bb0160d5483b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="고객관리" sheetId="1" r:id="R38d56b65b9194e2d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2760,33 +2760,7 @@
         <x:v>https://k-jewelry.kr/default/company/company_6.php?sub=04&amp;tit=01</x:v>
       </x:c>
     </x:row>
-    <x:row r="65">
-      <x:c r="A65" s="11" t="d">
-        <x:v>2026-10-20T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="B65" t="str">
-        <x:v>엠셀(Mcell)</x:v>
-      </x:c>
-      <x:c r="C65" t="str">
-        <x:v>경기 성남·안성</x:v>
-      </x:c>
-      <x:c r="D65" t="str">
-        <x:v>스마트웨어·발열 의류 OEM/ODM</x:v>
-      </x:c>
-      <x:c r="E65" t="str">
-        <x:v>contact@mcell.co.kr</x:v>
-      </x:c>
-      <x:c r="F65" t="str">
-        <x:v>070-4333-5233</x:v>
-      </x:c>
-      <x:c r="G65" t="str">
-        <x:v>발열 의류·스마트웨어 소재 개발 및 OEM/ODM</x:v>
-      </x:c>
-      <x:c r="H65" t="str">
-        <x:v>https://www.mcell.co.kr/mcell/oem-odm</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="65" s="9" customFormat="1" ht="14.4" customHeight="1">
+    <x:row r="65" s="9" customFormat="1" ht="14.399999618530273" customHeight="1">
       <x:c r="A65" s="11" t="n">
         <x:v>46307</x:v>
       </x:c>
@@ -2799,9 +2773,7 @@
       <x:c r="D65" t="str">
         <x:v>아동복 B2B 도매</x:v>
       </x:c>
-      <x:c r="E65" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="E65" t="str"/>
       <x:c r="F65" t="str">
         <x:v>010-6443-2599</x:v>
       </x:c>
@@ -2812,7 +2784,7 @@
         <x:v>https://www.sellernow.co.kr/post/501961</x:v>
       </x:c>
     </x:row>
-    <x:row r="66" s="9" customFormat="1" ht="14.4" customHeight="1">
+    <x:row r="66" s="9" customFormat="1" ht="14.399999618530273" customHeight="1">
       <x:c r="A66" s="11" t="n">
         <x:v>46307</x:v>
       </x:c>
@@ -2825,9 +2797,7 @@
       <x:c r="D66" t="str">
         <x:v>여성의류 B2B 도매</x:v>
       </x:c>
-      <x:c r="E66" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="E66" t="str"/>
       <x:c r="F66" t="str">
         <x:v>010-8780-0823</x:v>
       </x:c>
@@ -2838,7 +2808,7 @@
         <x:v>https://www.sellernow.co.kr/post/500851</x:v>
       </x:c>
     </x:row>
-    <x:row r="67" s="9" customFormat="1" ht="14.4" customHeight="1">
+    <x:row r="67" s="9" customFormat="1" ht="14.399999618530273" customHeight="1">
       <x:c r="A67" s="11" t="n">
         <x:v>46307</x:v>
       </x:c>
@@ -2851,9 +2821,7 @@
       <x:c r="D67" t="str">
         <x:v>여성의류 B2B 도매</x:v>
       </x:c>
-      <x:c r="E67" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="E67" t="str"/>
       <x:c r="F67" t="str">
         <x:v>010-4896-9951</x:v>
       </x:c>
@@ -2864,7 +2832,7 @@
         <x:v>https://ozbridge.co.kr/shopinfo/faq.html</x:v>
       </x:c>
     </x:row>
-    <x:row r="68" s="9" customFormat="1" ht="14.4" customHeight="1">
+    <x:row r="68" s="9" customFormat="1" ht="14.399999618530273" customHeight="1">
       <x:c r="A68" s="11" t="n">
         <x:v>46307</x:v>
       </x:c>
@@ -2877,9 +2845,7 @@
       <x:c r="D68" t="str">
         <x:v>아동복 B2B 도매</x:v>
       </x:c>
-      <x:c r="E68" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="E68" t="str"/>
       <x:c r="F68" t="str">
         <x:v>010-8113-2213</x:v>
       </x:c>
@@ -2890,7 +2856,7 @@
         <x:v>https://www.sellernow.co.kr/post/501960</x:v>
       </x:c>
     </x:row>
-    <x:row r="69" s="9" customFormat="1" ht="14.4" customHeight="1">
+    <x:row r="69" s="9" customFormat="1" ht="14.399999618530273" customHeight="1">
       <x:c r="A69" s="11" t="n">
         <x:v>46307</x:v>
       </x:c>
@@ -2903,9 +2869,7 @@
       <x:c r="D69" t="str">
         <x:v>아동복 자체제작·도매</x:v>
       </x:c>
-      <x:c r="E69" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="E69" t="str"/>
       <x:c r="F69" t="str">
         <x:v>010-6316-8732</x:v>
       </x:c>
@@ -2916,7 +2880,7 @@
         <x:v>https://sellernow.co.kr/post/502008</x:v>
       </x:c>
     </x:row>
-    <x:row r="70" s="9" customFormat="1" ht="14.4" customHeight="1">
+    <x:row r="70" s="9" customFormat="1" ht="14.399999618530273" customHeight="1">
       <x:c r="A70" s="11" t="n">
         <x:v>46307</x:v>
       </x:c>
@@ -2942,7 +2906,7 @@
         <x:v>https://www.luardmaison.co.kr/SECRETB2B</x:v>
       </x:c>
     </x:row>
-    <x:row r="71" s="9" customFormat="1" ht="14.4" customHeight="1">
+    <x:row r="71" s="9" customFormat="1" ht="14.399999618530273" customHeight="1">
       <x:c r="A71" s="11" t="n">
         <x:v>46307</x:v>
       </x:c>
@@ -2968,7 +2932,7 @@
         <x:v>https://funnydome.com/product/search.html</x:v>
       </x:c>
     </x:row>
-    <x:row r="72" s="9" customFormat="1" ht="14.4" customHeight="1">
+    <x:row r="72" s="9" customFormat="1" ht="14.399999618530273" customHeight="1">
       <x:c r="A72" s="11" t="n">
         <x:v>46307</x:v>
       </x:c>
@@ -2994,7 +2958,7 @@
         <x:v>https://maidome.com/goods/populate.php</x:v>
       </x:c>
     </x:row>
-    <x:row r="73" s="9" customFormat="1" ht="14.4" customHeight="1">
+    <x:row r="73" s="9" customFormat="1" ht="14.399999618530273" customHeight="1">
       <x:c r="A73" s="11" t="n">
         <x:v>46307</x:v>
       </x:c>
@@ -3020,7 +2984,7 @@
         <x:v>https://www.star-bag.com/store4</x:v>
       </x:c>
     </x:row>
-    <x:row r="74" s="9" customFormat="1" ht="14.4" customHeight="1">
+    <x:row r="74" s="9" customFormat="1" ht="14.399999618530273" customHeight="1">
       <x:c r="A74" s="11" t="n">
         <x:v>46307</x:v>
       </x:c>
@@ -3033,9 +2997,7 @@
       <x:c r="D74" t="str">
         <x:v>의류·패션잡화 B2B 도매</x:v>
       </x:c>
-      <x:c r="E74" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="E74" t="str"/>
       <x:c r="F74" t="str">
         <x:v>010-7708-2360</x:v>
       </x:c>
@@ -3044,6 +3006,260 @@
       </x:c>
       <x:c r="H74" t="str">
         <x:v>https://www.shinhan.ac.kr/bbs/kr/197/89939/download.do</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" t="str">
+        <x:v>2026-10-24</x:v>
+      </x:c>
+      <x:c r="B75" t="str">
+        <x:v>에이팩토리인터내셔널</x:v>
+      </x:c>
+      <x:c r="C75" t="str">
+        <x:v>서울 성북구</x:v>
+      </x:c>
+      <x:c r="D75" t="str">
+        <x:v>의류 OEM·ODM·원단·부자재</x:v>
+      </x:c>
+      <x:c r="E75" t="str">
+        <x:v>info@a-factory.co.kr</x:v>
+      </x:c>
+      <x:c r="F75" t="str">
+        <x:v>070-4417-6248</x:v>
+      </x:c>
+      <x:c r="G75" t="str">
+        <x:v>국내·중국 의류 생산 및 원부자재 소싱</x:v>
+      </x:c>
+      <x:c r="H75" t="str">
+        <x:v>https://a-factory.co.kr/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" t="str">
+        <x:v>2026-10-24</x:v>
+      </x:c>
+      <x:c r="B76" t="str">
+        <x:v>J&amp;G(모노디오)</x:v>
+      </x:c>
+      <x:c r="C76" t="str">
+        <x:v>경기 용인</x:v>
+      </x:c>
+      <x:c r="D76" t="str">
+        <x:v>스포츠웨어·기능성 원단</x:v>
+      </x:c>
+      <x:c r="E76" t="str">
+        <x:v>monodio@naver.com</x:v>
+      </x:c>
+      <x:c r="F76" t="str">
+        <x:v>010-6677-2441</x:v>
+      </x:c>
+      <x:c r="G76" t="str">
+        <x:v>국내 의류·원단 OEM/ODM 및 샘플 개발</x:v>
+      </x:c>
+      <x:c r="H76" t="str">
+        <x:v>https://jgapparel.co.kr/ko</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" t="str">
+        <x:v>2026-10-24</x:v>
+      </x:c>
+      <x:c r="B77" t="str">
+        <x:v>스와치온</x:v>
+      </x:c>
+      <x:c r="C77" t="str">
+        <x:v>서울 성동구</x:v>
+      </x:c>
+      <x:c r="D77" t="str">
+        <x:v>패션 원단·부자재</x:v>
+      </x:c>
+      <x:c r="E77" t="str">
+        <x:v>ask@swatchon.com</x:v>
+      </x:c>
+      <x:c r="F77" t="str">
+        <x:v>02-460-4200</x:v>
+      </x:c>
+      <x:c r="G77" t="str">
+        <x:v>동대문 원단 온라인 소싱 플랫폼</x:v>
+      </x:c>
+      <x:c r="H77" t="str">
+        <x:v>https://www.swatchon.com/help/contact</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78" t="str">
+        <x:v>2026-10-24</x:v>
+      </x:c>
+      <x:c r="B78" t="str">
+        <x:v>브랜딧</x:v>
+      </x:c>
+      <x:c r="C78" t="str">
+        <x:v>경기 양주시</x:v>
+      </x:c>
+      <x:c r="D78" t="str">
+        <x:v>브랜드 포장·택배봉투</x:v>
+      </x:c>
+      <x:c r="E78" t="str">
+        <x:v>with@brand-it.kr</x:v>
+      </x:c>
+      <x:c r="F78"/>
+      <x:c r="G78" t="str">
+        <x:v>온라인 브랜드용 포장재 직접 제조</x:v>
+      </x:c>
+      <x:c r="H78" t="str">
+        <x:v>https://www.brandit.kr/contacts</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79">
+      <x:c r="A79" t="str">
+        <x:v>2026-10-24</x:v>
+      </x:c>
+      <x:c r="B79" t="str">
+        <x:v>골라라</x:v>
+      </x:c>
+      <x:c r="C79" t="str">
+        <x:v>서울 동대문</x:v>
+      </x:c>
+      <x:c r="D79" t="str">
+        <x:v>K-패션 도매·수출</x:v>
+      </x:c>
+      <x:c r="E79" t="str">
+        <x:v>cs@gollala.me</x:v>
+      </x:c>
+      <x:c r="F79" t="str">
+        <x:v>02-6245-1111</x:v>
+      </x:c>
+      <x:c r="G79" t="str">
+        <x:v>동대문 패션 도매 글로벌 B2B 플랫폼</x:v>
+      </x:c>
+      <x:c r="H79" t="str">
+        <x:v>https://wowseattle.com/wow-posts/hot-deal-forum/294005/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80">
+      <x:c r="A80" t="str">
+        <x:v>2026-10-24</x:v>
+      </x:c>
+      <x:c r="B80" t="str">
+        <x:v>지비앤케이 인터내셔널</x:v>
+      </x:c>
+      <x:c r="C80" t="str">
+        <x:v>서울 마포구</x:v>
+      </x:c>
+      <x:c r="D80" t="str">
+        <x:v>의류 OEM·ODM·소싱</x:v>
+      </x:c>
+      <x:c r="E80" t="str">
+        <x:v>contact@gbkay.com</x:v>
+      </x:c>
+      <x:c r="F80" t="str">
+        <x:v>010-9443-4741</x:v>
+      </x:c>
+      <x:c r="G80" t="str">
+        <x:v>의류 생산·무역대행·소싱·물류</x:v>
+      </x:c>
+      <x:c r="H80" t="str">
+        <x:v>https://gbkay.com/production</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81">
+      <x:c r="A81" t="str">
+        <x:v>2026-10-24</x:v>
+      </x:c>
+      <x:c r="B81" t="str">
+        <x:v>연일섬유</x:v>
+      </x:c>
+      <x:c r="C81" t="str">
+        <x:v>서울 종로구·경기 포천</x:v>
+      </x:c>
+      <x:c r="D81" t="str">
+        <x:v>뜨개실·원사·니트 부자재</x:v>
+      </x:c>
+      <x:c r="E81" t="str">
+        <x:v>master@yeoniltex.com</x:v>
+      </x:c>
+      <x:c r="F81" t="str">
+        <x:v>02-2263-7117</x:v>
+      </x:c>
+      <x:c r="G81" t="str">
+        <x:v>뜨개실·원사 국내 개발·생산 및 ODM</x:v>
+      </x:c>
+      <x:c r="H81" t="str">
+        <x:v>https://www.yeoniltex.com/odm</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82">
+      <x:c r="A82" t="str">
+        <x:v>2026-10-24</x:v>
+      </x:c>
+      <x:c r="B82" t="str">
+        <x:v>JMONZ OEM ODM CREW</x:v>
+      </x:c>
+      <x:c r="C82" t="str">
+        <x:v>서울</x:v>
+      </x:c>
+      <x:c r="D82" t="str">
+        <x:v>의류 OEM·ODM·리빙소품</x:v>
+      </x:c>
+      <x:c r="E82" t="str">
+        <x:v>8911a@naver.com</x:v>
+      </x:c>
+      <x:c r="F82" t="str">
+        <x:v>02-555-3975</x:v>
+      </x:c>
+      <x:c r="G82" t="str">
+        <x:v>소량 의류 제작·OEM/ODM·판매 대행</x:v>
+      </x:c>
+      <x:c r="H82" t="str">
+        <x:v>https://jmonz.imweb.me/OEMODM</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83">
+      <x:c r="A83" t="str">
+        <x:v>2026-10-24</x:v>
+      </x:c>
+      <x:c r="B83" t="str">
+        <x:v>드림케이</x:v>
+      </x:c>
+      <x:c r="C83" t="str">
+        <x:v>서울 의류제조</x:v>
+      </x:c>
+      <x:c r="D83" t="str">
+        <x:v>우븐 의류·남녀정장·캐주얼·유니폼</x:v>
+      </x:c>
+      <x:c r="E83"/>
+      <x:c r="F83" t="str">
+        <x:v>010-5201-5649</x:v>
+      </x:c>
+      <x:c r="G83" t="str">
+        <x:v>서울 의류제조 봉제공장 공개 업체</x:v>
+      </x:c>
+      <x:c r="H83" t="str">
+        <x:v>https://www.ksct.or.kr/up_file/202208190303541806873.pdf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84">
+      <x:c r="A84" t="str">
+        <x:v>2026-10-24</x:v>
+      </x:c>
+      <x:c r="B84" t="str">
+        <x:v>가람패션</x:v>
+      </x:c>
+      <x:c r="C84" t="str">
+        <x:v>서울 의류제조</x:v>
+      </x:c>
+      <x:c r="D84" t="str">
+        <x:v>우븐·토털웨어</x:v>
+      </x:c>
+      <x:c r="E84"/>
+      <x:c r="F84" t="str">
+        <x:v>010-5334-4251</x:v>
+      </x:c>
+      <x:c r="G84" t="str">
+        <x:v>서울 의류제조 봉제공장 공개 업체</x:v>
+      </x:c>
+      <x:c r="H84" t="str">
+        <x:v>https://www.ksct.or.kr/up_file/202208190303541806873.pdf</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3053,7 +3269,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Radc65a55e2e249ea"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ddc6a6f34664656"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>